<commit_message>
feat(data): add real-world validation parts 9002 (Air Gripper) and 9003 (Clamp Cylinder) with STEP/IGES/PDF and Excel records
</commit_message>
<xml_diff>
--- a/docs/real_world/real_world_records.xlsx
+++ b/docs/real_world/real_world_records.xlsx
@@ -418,15 +418,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
-    <col width="33" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
     <col width="26" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
     <col width="53" customWidth="1" min="5" max="5"/>
-    <col width="44" customWidth="1" min="6" max="6"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
     <col width="36" customWidth="1" min="7" max="7"/>
     <col width="18" customWidth="1" min="8" max="8"/>
     <col width="22" customWidth="1" min="9" max="9"/>
@@ -553,6 +553,122 @@
       </c>
       <c r="L2" t="n">
         <v>20</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>9002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Wider Air Gripper HFT Series (HFT32)</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Aluminum 6061-T6</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>255 x 110 x 90 (billet block)</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>245 x 100 x 82 envelope; Bore Ø32, Stroke 60 mm</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Mounting holes M8x1.25, 4 x Ø4.2, 4 x Ø12 c-bore</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Haas VF-2 mill</t>
+        </is>
+      </c>
+      <c r="H3" t="n">
+        <v>42</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>±0.05 mm</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Ra 0.8</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Hard Anodize</t>
+        </is>
+      </c>
+      <c r="L3" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>9003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Clamp Cylinder MCK Series (MCK80)</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Aluminum 7075-T6</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>260 x 125 x 100 (billet block)</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>253 x 115 x 93 envelope; Bore Ø80, Stroke 75 mm</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Port threads PT 3/8, mounting M6x1</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Mazak Integrex e-420H</t>
+        </is>
+      </c>
+      <c r="H4" t="n">
+        <v>65</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>±0.05 mm</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Ra 0.8</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="L4" t="n">
+        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -566,13 +682,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
     <col width="7" customWidth="1" min="2" max="2"/>
-    <col width="32" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="48" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
@@ -770,6 +886,254 @@
         <v>4</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>9002</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>10</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Face 6 sides to envelope 245 x 100 x 82</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Haas VF-2</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Ø50 face mill</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>12</v>
+      </c>
+      <c r="G7" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>9002</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>20</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Bore Ø32 cylinder chamber</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Haas VF-2</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Ø20 boring head</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>6</v>
+      </c>
+      <c r="G8" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>9002</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>30</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Mill guide tracks and pockets</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Haas VF-2</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Ø12 end mill</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>8</v>
+      </c>
+      <c r="G9" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>9002</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>40</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Drill and tap M8x1.25 / M10x1.5 mounting holes</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Haas VF-2</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Ø6.8 drill, M8 tap</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>5</v>
+      </c>
+      <c r="G10" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>9003</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>10</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Rough turn OD and face cylinder body</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Mazak Integrex</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>CNMG 120408 insert</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>15</v>
+      </c>
+      <c r="G11" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>9003</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>20</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Finish bore Ø80 cylinder cavity</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Mazak Integrex</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Ø50 boring bar</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>10</v>
+      </c>
+      <c r="G12" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>9003</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>30</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Thread port holes PT 3/8</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Mazak Integrex</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>PT 3/8 tap</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>8</v>
+      </c>
+      <c r="G13" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>9003</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>40</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Mill clamp mounting brackets and pockets</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Mazak Integrex</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Ø16 end mill</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>12</v>
+      </c>
+      <c r="G14" t="n">
+        <v>14</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(data): add real-world validation parts 9004 (Bevel Gear), 9005 (Bearing Bracket), 9006 (Stepped Shaft) with STEP/IGES and Excel records
</commit_message>
<xml_diff>
--- a/docs/real_world/real_world_records.xlsx
+++ b/docs/real_world/real_world_records.xlsx
@@ -418,20 +418,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
     <col width="38" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="53" customWidth="1" min="5" max="5"/>
-    <col width="50" customWidth="1" min="6" max="6"/>
-    <col width="36" customWidth="1" min="7" max="7"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="51" customWidth="1" min="6" max="6"/>
+    <col width="48" customWidth="1" min="7" max="7"/>
     <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="22" customWidth="1" min="9" max="9"/>
-    <col width="24" customWidth="1" min="10" max="10"/>
-    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="29" customWidth="1" min="9" max="9"/>
+    <col width="33" customWidth="1" min="10" max="10"/>
+    <col width="27" customWidth="1" min="11" max="11"/>
     <col width="11" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
@@ -669,6 +669,180 @@
       </c>
       <c r="L4" t="n">
         <v>30</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>9004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Helical Bevel Gear</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>20MnCr5 alloy steel</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Ø180 x 305 forging</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>295 x 170 x 170 envelope; centre bore Ø25, teeth pitch dia Ø170</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Centre bore Ø25, 2 x Ø20 radial pin holes</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Mazak QT-200 lathe, Gleason CNC gear generator</t>
+        </is>
+      </c>
+      <c r="H5" t="n">
+        <v>48</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>±0.02 mm (DIN 3962 Class 6)</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Ra 0.8 ground teeth</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Case carburized 58-62 HRC</t>
+        </is>
+      </c>
+      <c r="L5" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>9005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Bearing Bracket Flanged Pivot Mount</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Ductile Iron EN-GJS-400-15</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>200 x 270 x 240 casting</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>192 x 258.5 x 229.5 envelope; bearing bore Ø45, 4 flange holes</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>4 x Ø20 through on flange; 2 x Ø10 alignment pins</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Haas VF-4 4-axis mill</t>
+        </is>
+      </c>
+      <c r="H6" t="n">
+        <v>38</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>±0.05 mm</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Ra 1.6 (Ra 0.8 in bearing bore)</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Stress relieved</t>
+        </is>
+      </c>
+      <c r="L6" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>9006</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Wind Turbine Main Shaft</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>42CrMo4 alloy steel</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Ø105 x 205 forging</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Ø96 x 190 overall; step diameters Ø96, Ø24, Ø16</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>None (centre turned)</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Mazak QT-350 CNC lathe</t>
+        </is>
+      </c>
+      <c r="H7" t="n">
+        <v>25</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>±0.03 mm</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Ra 0.8 bearing seats</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Quenched and tempered</t>
+        </is>
+      </c>
+      <c r="L7" t="n">
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -682,14 +856,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:G22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
     <col width="7" customWidth="1" min="2" max="2"/>
     <col width="48" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="27" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
   </cols>
@@ -1134,6 +1308,254 @@
         <v>14</v>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>9004</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>10</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Turn blank OD and bore Ø25</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Mazak QT-200</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>CNMG 120408, boring bar</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>10</v>
+      </c>
+      <c r="G15" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>9004</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>20</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Generate spiral bevel gear teeth</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Gleason CNC</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Bevel cutter head</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>15</v>
+      </c>
+      <c r="G16" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>9004</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>30</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Drill 2 x Ø20 radial pin holes</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Haas VF-2</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Ø20 drill</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>5</v>
+      </c>
+      <c r="G17" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>9005</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>10</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Face base flange and mill mounting pads</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Haas VF-4</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Ø80 face mill</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
+        <v>8</v>
+      </c>
+      <c r="G18" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>9005</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>20</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Drill 4 flange holes Ø20</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Haas VF-4</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Ø20 carbide drill</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
+        <v>6</v>
+      </c>
+      <c r="G19" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>9005</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>30</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Bore Ø45 bearing journal and Ø75 recess</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Haas VF-4</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Precision boring head</t>
+        </is>
+      </c>
+      <c r="F20" t="n">
+        <v>8</v>
+      </c>
+      <c r="G20" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>9006</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>10</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Rough and finish turn Ø96, Ø24, Ø16 steps</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Mazak QT-350</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>CNMG 120408 / VNMG 160404</t>
+        </is>
+      </c>
+      <c r="F21" t="n">
+        <v>10</v>
+      </c>
+      <c r="G21" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>9006</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>20</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Grind bearing journals to Ra 0.8</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Studer cylindrical grinder</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Al2O3 grinding wheel</t>
+        </is>
+      </c>
+      <c r="F22" t="n">
+        <v>8</v>
+      </c>
+      <c r="G22" t="n">
+        <v>7</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(data): add real-world validation parts 9007 (MG996 Servo Bracket) and 9008 (Pivot Support Fork Clevis Bracket)
</commit_message>
<xml_diff>
--- a/docs/real_world/real_world_records.xlsx
+++ b/docs/real_world/real_world_records.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:L9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -426,12 +426,12 @@
     <col width="28" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="51" customWidth="1" min="6" max="6"/>
+    <col width="57" customWidth="1" min="6" max="6"/>
     <col width="48" customWidth="1" min="7" max="7"/>
     <col width="18" customWidth="1" min="8" max="8"/>
     <col width="29" customWidth="1" min="9" max="9"/>
     <col width="33" customWidth="1" min="10" max="10"/>
-    <col width="27" customWidth="1" min="11" max="11"/>
+    <col width="41" customWidth="1" min="11" max="11"/>
     <col width="11" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
@@ -843,6 +843,122 @@
       </c>
       <c r="L7" t="n">
         <v>15</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>9007</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>MG996 Servo Bracket</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Aluminum 6061-T6</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>65 x 45 x 30 (extruded block)</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>57.2 x 39.1 x 26.0 envelope</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>8 x Ø4.2 mounting holes, 2 x Ø2.0 locator holes</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Haas Mini Mill</t>
+        </is>
+      </c>
+      <c r="H8" t="n">
+        <v>16</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>±0.1 mm</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Ra 1.6</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Black Anodized</t>
+        </is>
+      </c>
+      <c r="L8" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>9008</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Pivot Support Clevis Bracket</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>AISI 1045 steel</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>165 x 50 x 135 forging blank</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>156.3 x 40.0 x 123.9 envelope; 40 mm clevis fork width</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>2 x Ø20 pivot holes; 1 x Ø16 mount hole; 1 x Ø12.5 hole</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Haas VF-3 mill</t>
+        </is>
+      </c>
+      <c r="H9" t="n">
+        <v>34</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>±0.05 mm</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Ra 1.6 (Ra 0.8 pivot bore)</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Induction harden pivot bore (50-54 HRC)</t>
+        </is>
+      </c>
+      <c r="L9" t="n">
+        <v>40</v>
       </c>
     </row>
   </sheetData>
@@ -856,7 +972,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G22"/>
+  <dimension ref="A1:G28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1556,6 +1672,192 @@
         <v>7</v>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>9007</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>10</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Mill perimeter profile and servo pocket</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Haas Mini Mill</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Ø6 carbide end mill</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>6</v>
+      </c>
+      <c r="G23" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>9007</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>20</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Drill 8 x Ø4.2 and 2 x Ø2.0 holes</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Haas Mini Mill</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Ø4.2 drill, Ø2.0 drill</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
+        <v>4</v>
+      </c>
+      <c r="G24" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>9008</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>10</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Face mill top, bottom and fork cheeks</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Haas VF-3</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Ø63 face mill</t>
+        </is>
+      </c>
+      <c r="F25" t="n">
+        <v>10</v>
+      </c>
+      <c r="G25" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>9008</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>20</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Mill central clevis slot width 40 mm</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Haas VF-3</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Ø25 roughing end mill</t>
+        </is>
+      </c>
+      <c r="F26" t="n">
+        <v>8</v>
+      </c>
+      <c r="G26" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>9008</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>30</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Drill and bore 2 x Ø20 pivot holes</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Haas VF-3</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Ø20 drill and boring head</t>
+        </is>
+      </c>
+      <c r="F27" t="n">
+        <v>6</v>
+      </c>
+      <c r="G27" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>9008</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>40</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Drill Ø16 mounting hole and Ø12.5 hole</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Haas VF-3</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Ø16 drill, Ø12.5 drill</t>
+        </is>
+      </c>
+      <c r="F28" t="n">
+        <v>5</v>
+      </c>
+      <c r="G28" t="n">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>